<commit_message>
Validation: fill batch 2 (30 clips, all 15 dialects) + merged 61-clip human-validation file
</commit_message>
<xml_diff>
--- a/evaluation/results/validation_sample.xlsx
+++ b/evaluation/results/validation_sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Niloy Islam PhD\ASR work bengali\evaluation\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD692D81-96E3-4A27-A00F-D88F6C6DD88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A10F8A18-FE09-4AD2-A184-D0FC46942E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1037" uniqueCount="648">
   <si>
     <t>clip_id</t>
   </si>
@@ -1894,6 +1894,81 @@
   </si>
   <si>
     <t>দারিকাড়া তোয়লো ইতিলা পোষদ আউতেল আনিগে বড়ে উল্লা তুরকা নান্দন অব্য়</t>
+  </si>
+  <si>
+    <t>সেগুনের ছায়ায় দাঁড়িয়ে মুক্ত মঞ্চে শিক্ষার্থীদের সাংস্কৃতিক বিকাশের পরিচায়ক।</t>
+  </si>
+  <si>
+    <t>কি জানির মত সাদা হয়ে গেছে, কি যে গন্ধ আমি তহ কিছু বুঝতে পারতাছি না সো মাননীয় একাহ্নে প্রমান করার কিছুই নেই মাননীয়মন্ডল , ধন্যবাদ সবাইকে । জমে গেছে জেলার বিতর্ক</t>
+  </si>
+  <si>
+    <t xml:space="preserve">এই সাকসেসটা আমার জন্য আশীর্বাদ। এই পরিচয়টা দিয়ে উনি খুব সাছন্দ্যবোধ করতেন এবং খুবি এটাকে প্রাইড আকারে নিতেন  তো আমার মনে হয় না উনি আহংকারি ছিলেন এবং আমার কাছে মনে হয় যে উনিও খুব কষ্ট করেছেন , একটা সময়ে সে কষ্ট </t>
+  </si>
+  <si>
+    <t xml:space="preserve">আমি এরকম অনেক মানুষকে চিনি যারা  হচ্ছে mood যখন off থাকে তাদের একটু হাসির দরকার হয় , তারা চিটাগনিয়ান নাটকগুলা দেখে, চিটাগিনিয়ান language যেগুলি সেগুলা দেখে তারা তাদের mood refresh করে। চট্রগ্রামের ভাষাটাই unique . </t>
+  </si>
+  <si>
+    <t xml:space="preserve">এগুলা কি আমরা চোখে দেখতে পাবো , রাস্তার ডানপাশের এই বিল্ডিংটা হচ্ছে কৃষি বিপণন ভবন রংপুর , গোলচত্তর কেন জেনো আমার কাছে ভালো লেগেছে , বাঘের মুর্তি, তহ ফাইনালি </t>
+  </si>
+  <si>
+    <t>alright আমাদের exciting Rapid Fire রাউন্ডটি কিন্তু শেষ হয়ে গেছে, ওয়ে already have the score, আদমজী ক্যান্টেন্মেন্ট কলেজের স্কোর হচ্ছে টোটাল 8  কারণ তাদের কিন্তু দুইটো ভুল হয়েছিল এবং ভিকাউননেসা স্কুল এন্ড কলেজ কিন্তু সবগুলা</t>
+  </si>
+  <si>
+    <t>আসসালাইমুয়ালাইকুম টু everyone গাইজ, This is your boy আবির হাসান, Welcome to my channel , Welcome to another video এবং এটা হতে যাচ্ছে আমার মিশন রংপুর ডিবিশনের second video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">একটা কথা চিন্তা করছেন কি, এহন যদি কথাটা না কই আর পোলাটার কাক্কা পরে কিন্তু আমগই দোষবো , জাইন্না শুইন্যা কথাটা কস নাই কা । এই কি হইছে আমারে কউ না কা , হুদাই আমারে tension এ ফালাইতাছো </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohammad Ali, am from bangladesh in sylhet. so sylhet is your hometown. yeag yeah, my motherland sylhet.i born this . what are you doing now  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">আব হামারি সাধীকো দু শাল হো জুকি হে  , সেক্স কা বাদ তহ ওটিপি মাং তা হেয় গান্ডু । দিক্কাত হে  ইয়ার </t>
+  </si>
+  <si>
+    <t xml:space="preserve">বর্তমানে আমি আছি বরিশাল ইউনিভার্সিটি </t>
+  </si>
+  <si>
+    <t xml:space="preserve">কি হইছে রে , আস্তে চালাইতে পারেন না , দেখে চালান </t>
+  </si>
+  <si>
+    <t>কে কিতা কইলো ,ইতান আমি হুনাত নাই , আচ্ছা হুনি যাও , ভাই আয়ো আয়ো . হুবাযায় হুবাযায় খাপ দরখাডি মাত মাতিলে আছা হোসা, একো সামনে আইনাখে মুবাইলে হোতারাক সিলি</t>
+  </si>
+  <si>
+    <t xml:space="preserve">বর্তমান  বাংলাদেশ মাতাইলাইছে কেলা ? আরেফিন শুভ, ইতারাও কিন্তু আমাদের দেশের ছেড়া এন্ড ছেড়ি , আপনাদের মনে একটা প্রইশ্ন আইসতে পারে না বর্তমান বাংলাদেশের ছেড়াছেড়িরা এই ময়মনসিং এর ছেলেদের বিয়ে করার জন্য এত উতাল মাতাল  কি জইন্যে, জাইনুন </t>
+  </si>
+  <si>
+    <t>এই দ্বীপটির সৌন্দর্য আসলে ভাষায় প্রকাশ করার মতো নয়। আপনি যদি বরিশালে আসেন, অবশ্যই এই দুর্গে সাগর দেখে যাবেন। চলুন, এই দুর্গে সাগরের মনোমুগ্ধকর দৃশ্যগুলোকে সিনেমাটিক শটের মাধ্যমে দেখে আসি</t>
+  </si>
+  <si>
+    <t>আপনাদের লাইগ্যা ময়মনসিংয়ের ভাষায় কথা বলার চেষ্টা করলাম। ভুলত্রুটি  করলে ক্ষমাসুন্দর  দৃষ্টিতে দেখবেন আপনারা। কিতা হয়েছে তোমরা নাচতেছো না কেনো , এখানে আসো তুমি , এখানে এসে নাচো , এইতো ঠিক আছে, এভাবেই দুলাইতে হবে</t>
+  </si>
+  <si>
+    <t>এই ক্ষেত্রে আমার সত্যিই  একটু জিজ্ঞাসা রয়েছে । আমার মনে হচ্ছে, কোনো পরিচিত মানুষ  বা অন্য কোনো মানুষকে বা তাদের কোন গেস্টকে  লেগ  পুল করে দেবে</t>
+  </si>
+  <si>
+    <t>ইতে পুর্বে তুমি খেয়ারে বহু দুকা দিসো, বহু মিত্যা কথা বলসো, প্রবঞ্ছনা করসো, ইতো ভুলা তুমি সাইদো না ফহিন্নি , আপনে কথা  যেইদডা কোই ছুইন যে কথাডা বোলেছেন আপনে এটা কিন্তু েকদম খাটি কথা</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> তোমাদের কয়লাসুন্দরের মত নাইচা দেখাই  এই যে ভাবে গুইরা তারপরে নাচা শেষ করতে হবে, আস্তে আস্তে কইরা  কোমর দুলাইতে হবে কিন্তু আমিতো পারি না কয়লা সুন্দরীর   মতন নাচতে, আমি তহ সব সময় এভাবেই নাচি </t>
+  </si>
+  <si>
+    <t>কিন্তু আপনারা সবাই একসতে , হে আমিছে আপনে আতো জোর ধাক্কা দিলেন কি জন্যে  যদি  কোমর এমনে থামাইতাম ? এতো জুরে কওয়ার কি আছে ?  বেলা কারা ছিলো Sorry ভাই  Sorry</t>
+  </si>
+  <si>
+    <t>মানে, বুদ্ধিগুলো শিখার জন্য। এই যে, এগুলা আমি শিখতে শিখতে আজকে  ইনশাল্লাহ ব্যবসা করতে পারি । আমার সবকিছু চলতেছে ইনশাল্লাহ আল্লাহর রহমতে।  তো ভাষা  শিখার পাশাপাশে তোমার বাংলারদেশে যাবার ইচ্ছা নেই।</t>
+  </si>
+  <si>
+    <t>একটির পর একটি নার্তকে হেলতে করে, এর পর কনা হামরোর সঙ্গে নার্তকে দেখা হয়। সেখানে ওরা একে অপরকে সেক্সি জুতো দেখায়। নার্তকে কনা হামরোর সেক্সি জুতো দেখে ইমপ্রুভ হয়, অনেক প্রাউট ফিল করে, কিন্তু সাকোরা ডিজগাস্টেড হয়। মারামারি শুরু করে</t>
+  </si>
+  <si>
+    <t xml:space="preserve">এটা আমার ফাজ ব্লগ করচ্চি আমি, বেশি বেশি করে আমাকে ভালোবাসা দিও , পাশে থেকে লাইক করো, সাবস্ক্রাইব কইরো, শেয়ার কইরো </t>
+  </si>
+  <si>
+    <t>দিস ওর কামিং আপ অন ইউর লেফট ইজ দিস</t>
+  </si>
+  <si>
+    <t xml:space="preserve">প্রিপজিশনের নিয়ম অনুসারে in the bus হওয়ার কথা বাট আমরা তহ in the bus  বলি না , আমরা বলি on the bus । ব্যাসিক্যালি আপনি যখন বাসে ট্রাভেল করেন  বা কোন যানবাহনে ট্রাভেল করেন on ব্যাবহার করি ঠিক সেইম ভাবে এরকম অনেক </t>
   </si>
 </sst>
 </file>
@@ -2302,7 +2377,9 @@
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3" t="s">
+        <v>623</v>
+      </c>
     </row>
     <row r="3" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2320,7 +2397,9 @@
       <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>624</v>
+      </c>
     </row>
     <row r="4" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -2338,7 +2417,9 @@
       <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="3"/>
+      <c r="F4" s="3" t="s">
+        <v>625</v>
+      </c>
     </row>
     <row r="5" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -2356,7 +2437,9 @@
       <c r="E5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="3"/>
+      <c r="F5" s="3" t="s">
+        <v>626</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -2374,9 +2457,11 @@
       <c r="E6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="F6" s="3" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2392,7 +2477,9 @@
       <c r="E7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>627</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -2410,7 +2497,9 @@
       <c r="E8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>629</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -2428,7 +2517,9 @@
       <c r="E9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>630</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -2446,7 +2537,9 @@
       <c r="E10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -2464,7 +2557,9 @@
       <c r="E11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>632</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -2482,7 +2577,9 @@
       <c r="E12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>633</v>
+      </c>
     </row>
     <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -2500,7 +2597,9 @@
       <c r="E13" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -2518,7 +2617,9 @@
       <c r="E14" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>635</v>
+      </c>
     </row>
     <row r="15" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -2536,7 +2637,9 @@
       <c r="E15" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>636</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -2554,7 +2657,9 @@
       <c r="E16" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="17" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -2572,9 +2677,11 @@
       <c r="E17" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F17" s="3"/>
-    </row>
-    <row r="18" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="F17" s="3" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>65</v>
       </c>
@@ -2590,7 +2697,9 @@
       <c r="E18" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F18" s="3"/>
+      <c r="F18" s="3" t="s">
+        <v>638</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -2608,7 +2717,9 @@
       <c r="E19" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F19" s="3"/>
+      <c r="F19" s="3" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -2626,7 +2737,9 @@
       <c r="E20" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F20" s="3"/>
+      <c r="F20" s="3" t="s">
+        <v>639</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -2644,7 +2757,9 @@
       <c r="E21" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F21" s="3"/>
+      <c r="F21" s="3" t="s">
+        <v>640</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -2662,7 +2777,9 @@
       <c r="E22" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F22" s="3"/>
+      <c r="F22" s="3" t="s">
+        <v>641</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
@@ -2680,7 +2797,9 @@
       <c r="E23" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -2698,9 +2817,11 @@
       <c r="E24" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F24" s="3"/>
-    </row>
-    <row r="25" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="F24" s="3" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>88</v>
       </c>
@@ -2716,7 +2837,9 @@
       <c r="E25" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F25" s="3"/>
+      <c r="F25" s="3" t="s">
+        <v>643</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -2734,7 +2857,9 @@
       <c r="E26" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F26" s="3"/>
+      <c r="F26" s="3" t="s">
+        <v>644</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -2752,7 +2877,9 @@
       <c r="E27" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F27" s="3"/>
+      <c r="F27" s="3" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="28" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -2770,7 +2897,9 @@
       <c r="E28" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F28" s="3"/>
+      <c r="F28" s="3" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -2788,7 +2917,9 @@
       <c r="E29" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F29" s="3"/>
+      <c r="F29" s="3" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -2806,7 +2937,9 @@
       <c r="E30" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F30" s="3"/>
+      <c r="F30" s="3" t="s">
+        <v>646</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -2824,9 +2957,11 @@
       <c r="E31" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="F31" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>112</v>
       </c>
@@ -2842,7 +2977,9 @@
       <c r="E32" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F32" s="3"/>
+      <c r="F32" s="3" t="s">
+        <v>647</v>
+      </c>
     </row>
     <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" t="s">

</xml_diff>